<commit_message>
Fix mobile layout and receipt formatting
</commit_message>
<xml_diff>
--- a/backend/Sales_Report.xlsx
+++ b/backend/Sales_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,6 +478,456 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:24:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hebba Cake</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>200</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:26:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>150</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:30:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:31:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Chocolate Affogato</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>160</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:36:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>150</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:37:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Chocolate Affogato</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>160</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:53:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>150</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:53:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>200</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-15 20:56:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:03:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>150</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:03:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Amour Sour Cherry</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>360</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:07:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Salankatia</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>200</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:07:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Nutella</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>150</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:07:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lava Cake</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>75</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:07:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brownie</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>75</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:07:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>150</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:09:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cheese Bomb</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>200</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:09:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>200</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:09:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>200</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:10:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cheese Bomb</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>200</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:10:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hebba Cake</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>200</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:10:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hebba Cake</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>200</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:10:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>200</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:11:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>150</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:11:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>150</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:11:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>200</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:14:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>150</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:14:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Classic Affogato</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>150</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:16:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Fazia Cake</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>200</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-03-15 21:16:51</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
changed the ui to be responsive
</commit_message>
<xml_diff>
--- a/backend/Sales_Report.xlsx
+++ b/backend/Sales_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,36 @@
           <t>date_date_timestamp</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Invoice No</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Item Name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Line Total</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -447,6 +477,12 @@
           <t>2026-03-15 11:33:12</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -462,6 +498,12 @@
           <t>2026-03-15 11:33:21</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -477,6 +519,12 @@
           <t>2026-03-15 11:46:04</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -492,6 +540,12 @@
           <t>2026-03-15 20:24:04</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -507,6 +561,12 @@
           <t>2026-03-15 20:26:52</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -522,6 +582,12 @@
           <t>2026-03-15 20:30:58</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -537,6 +603,12 @@
           <t>2026-03-15 20:31:57</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -552,6 +624,12 @@
           <t>2026-03-15 20:36:01</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -567,6 +645,12 @@
           <t>2026-03-15 20:37:01</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -582,6 +666,12 @@
           <t>2026-03-15 20:53:03</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -597,6 +687,12 @@
           <t>2026-03-15 20:53:03</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -612,6 +708,12 @@
           <t>2026-03-15 20:56:08</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -627,6 +729,12 @@
           <t>2026-03-15 21:03:14</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -642,6 +750,12 @@
           <t>2026-03-15 21:03:24</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -657,6 +771,12 @@
           <t>2026-03-15 21:07:42</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -672,6 +792,12 @@
           <t>2026-03-15 21:07:42</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -687,6 +813,12 @@
           <t>2026-03-15 21:07:42</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -702,6 +834,12 @@
           <t>2026-03-15 21:07:42</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -717,6 +855,12 @@
           <t>2026-03-15 21:07:42</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -732,6 +876,12 @@
           <t>2026-03-15 21:09:53</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -747,6 +897,12 @@
           <t>2026-03-15 21:09:53</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -762,6 +918,12 @@
           <t>2026-03-15 21:09:53</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -777,6 +939,12 @@
           <t>2026-03-15 21:10:02</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -792,6 +960,12 @@
           <t>2026-03-15 21:10:02</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -807,6 +981,12 @@
           <t>2026-03-15 21:10:22</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -822,6 +1002,12 @@
           <t>2026-03-15 21:10:43</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -837,6 +1023,12 @@
           <t>2026-03-15 21:11:01</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -852,6 +1044,12 @@
           <t>2026-03-15 21:11:18</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -867,6 +1065,12 @@
           <t>2026-03-15 21:11:36</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -882,6 +1086,12 @@
           <t>2026-03-15 21:14:52</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -897,6 +1107,12 @@
           <t>2026-03-15 21:14:52</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -912,6 +1128,12 @@
           <t>2026-03-15 21:16:04</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -927,6 +1149,127 @@
           <t>2026-03-15 21:16:51</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>84</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-03-23 07:39:58 PM</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Classic Affagato </t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="n">
+        <v>160</v>
+      </c>
+      <c r="I35" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>84</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-03-23 07:39:58 PM</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>85</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-03-23 07:40:11 PM</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Classic -cinnamon roll</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="n">
+        <v>200</v>
+      </c>
+      <c r="I37" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="n">
+        <v>85</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-03-23 07:40:11 PM</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fixed the ui issue
</commit_message>
<xml_diff>
--- a/backend/Sales_Report.xlsx
+++ b/backend/Sales_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1686,12 +1686,247 @@
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
+      <c r="D55" t="n">
+        <v>97</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:01 AM</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Oreo -cinnamon roll</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>220</v>
+      </c>
+      <c r="I55" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="n">
+        <v>97</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:01 AM</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="n">
+        <v>98</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:05 AM</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Oreo -cinnamon roll</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="n">
+        <v>220</v>
+      </c>
+      <c r="I57" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="n">
+        <v>98</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:05 AM</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="n">
+        <v>99</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:08 AM</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Coffee brulee</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="n">
+        <v>150</v>
+      </c>
+      <c r="I59" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="n">
+        <v>99</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:08 AM</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="n">
+        <v>100</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:13 AM</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salted caramel coffee </t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" t="n">
+        <v>150</v>
+      </c>
+      <c r="I61" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="n">
+        <v>100</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:13 AM</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Coffee brulee</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" t="n">
+        <v>150</v>
+      </c>
+      <c r="I62" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="n">
+        <v>100</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:18:13 AM</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>